<commit_message>
DA : colonne Unité (formulaire, import, PDF, Excel) ; colonne Seuil masquée
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A5nFHKBNu16d3KnVC8b1NF
</commit_message>
<xml_diff>
--- a/modeles/Canevas_DA.xlsx
+++ b/modeles/Canevas_DA.xlsx
@@ -1,26 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\OneDrive\Desktop\CANVA FILTRES\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEFB2801-D1CA-45BC-8491-2EACBE66D64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{254299C2-95CE-463A-B9B1-FC887C77F09C}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="31549" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="31549" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
-    <externalReference r:id="rId3"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'31549'!$A$1:$G$7</definedName>
     <definedName name="_xlcn.WorksheetConnection_Classeur4Tableau1" hidden="1">#REF!</definedName>
     <definedName name="_xlcn.WorksheetConnection_Classeur4Tableau11" hidden="1">#REF!</definedName>
     <definedName name="po" hidden="1">#REF!</definedName>
@@ -28,107 +20,64 @@
     <definedName name="Segment_CHANTIERS">#N/A</definedName>
     <definedName name="Segment_Engin">#N/A</definedName>
     <definedName name="TitreColonne1">[2]!Données[[#Headers],[Centre de coûts]]</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'31549'!$A$1:$H$7</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>DA</t>
-  </si>
-  <si>
-    <t>Désignation Catalogue</t>
-  </si>
-  <si>
-    <t>Quantité</t>
-  </si>
-  <si>
-    <t>Référance</t>
-  </si>
-  <si>
-    <t>Code_Engin</t>
-  </si>
-  <si>
-    <t>N° Poste</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="7">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -187,37 +136,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -228,8 +177,8 @@
     <dxf>
       <font>
         <condense val="0"/>
+        <color rgb="FF9C0006"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
@@ -240,8 +189,8 @@
     <dxf>
       <font>
         <condense val="0"/>
+        <color rgb="FF9C0006"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
@@ -251,23 +200,80 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="31549"/>
       <sheetName val="Etat de panne  a jour"/>
@@ -293,11 +299,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Données de coût et graphique"/>
       <sheetName val="Consommation Dhuile10"/>
@@ -620,108 +623,137 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7F81306-EBBE-4604-80CB-458CEDF573E8}">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.453125" defaultRowHeight="18.9" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.36328125" style="10" customWidth="1"/>
-    <col min="2" max="2" width="11" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="10" customWidth="1"/>
-    <col min="4" max="4" width="32.453125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.7265625" style="11" customWidth="1"/>
-    <col min="6" max="6" width="8.08984375" style="12" customWidth="1"/>
-    <col min="7" max="7" width="15" style="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.453125" style="8"/>
+    <col width="8.36328125" customWidth="1" style="10" min="1" max="1"/>
+    <col width="11" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
+    <col width="11" customWidth="1" style="10" min="3" max="3"/>
+    <col width="32.453125" bestFit="1" customWidth="1" style="11" min="4" max="4"/>
+    <col width="17.7265625" customWidth="1" style="11" min="5" max="5"/>
+    <col width="8.08984375" customWidth="1" style="12" min="6" max="6"/>
+    <col width="8" bestFit="1" customWidth="1" style="12" min="7" max="7"/>
+    <col width="15" customWidth="1" style="8" min="8" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" ht="18.9" customFormat="1" customHeight="1" s="3">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>DA</t>
+        </is>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>6</v>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>N° Poste</t>
+        </is>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Désignation Catalogue</t>
+        </is>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Référance</t>
+        </is>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>3</v>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Unité</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Code_Engin</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+    <row r="2" ht="18.9" customHeight="1">
+      <c r="A2" s="4" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
     </row>
-    <row r="3" spans="1:7" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+    <row r="3" ht="18.9" customHeight="1">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
     </row>
-    <row r="4" spans="1:7" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+    <row r="4" ht="18.9" customHeight="1">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
     </row>
-    <row r="5" spans="1:7" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+    <row r="5" ht="18.9" customHeight="1">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
     </row>
-    <row r="6" spans="1:7" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+    <row r="6" ht="18.9" customHeight="1">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
     </row>
-    <row r="7" spans="1:7" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+    <row r="7" ht="18.9" customHeight="1">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G7" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
+  <autoFilter ref="A1:H7"/>
   <conditionalFormatting sqref="B2:C7">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="ENCOURS">
+    <cfRule type="containsText" priority="1" operator="containsText" dxfId="0" text="ENCOURS">
       <formula>NOT(ISERROR(SEARCH("ENCOURS",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D8:E1048576 D1:E1">
-    <cfRule type="duplicateValues" dxfId="0" priority="7"/>
+  <conditionalFormatting sqref="D1:E1 D8:E1048576">
+    <cfRule type="duplicateValues" priority="7" dxfId="0"/>
   </conditionalFormatting>
-  <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.55118110236220474" bottom="0.55118110236220474" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="95" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.3149606299212598" right="0.3149606299212598" top="0.5511811023622047" bottom="0.5511811023622047" header="0.3149606299212598" footer="0.3149606299212598"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="95"/>
 </worksheet>
 </file>
</xml_diff>